<commit_message>
change to input file Fic Reg -adjustment
</commit_message>
<xml_diff>
--- a/data/Renal_Modelling_Input_File - Fictional Region.xlsx
+++ b/data/Renal_Modelling_Input_File - Fictional Region.xlsx
@@ -8,7 +8,8 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucy.Morgan\Desktop\Renal Modelling\simPy model\renal-capacity-model\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE615263-C5E6-449A-ACD1-DFDFB60FA202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC87F2B2-2F7F-4FDB-A5FE-C04D125920AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="dMegnNnE+zyybPgVIWqzEkMQijGQ93uCy4aeBHcIT4Ejq+vOTcmKp1h7/9ffuQ3mPj+vzBMv7Zi8FqaF4KYWZQ==" workbookSaltValue="OwdSQ8BfAne0ow/MYs2mig==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="823" activeTab="6" xr2:uid="{F2F90EEA-FE26-47F0-942A-1DBACAA9371D}"/>
   </bookViews>
@@ -35,9 +36,6 @@
     <sheet name="TxType" sheetId="10956" state="hidden" r:id="rId20"/>
     <sheet name="receivesTx" sheetId="11032" state="hidden" r:id="rId21"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId22"/>
-  </externalReferences>
   <definedNames>
     <definedName name="IncCCD1">'Scenario Inputs'!$G$61</definedName>
     <definedName name="IncCCD2">'Scenario Inputs'!$G$62</definedName>
@@ -1666,108 +1664,14 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="5" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="9" fontId="9" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1799,17 +1703,102 @@
     <xf numFmtId="9" fontId="6" fillId="3" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="5" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -1820,8 +1809,23 @@
     <xf numFmtId="2" fontId="8" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1829,19 +1833,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="20" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1852,29 +1860,46 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1907,65 +1932,38 @@
     <xf numFmtId="0" fontId="20" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="14" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="14" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -24824,144 +24822,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Cover Sheet"/>
-      <sheetName val="Background"/>
-      <sheetName val="DES Pathway Map"/>
-      <sheetName val="Costing Map"/>
-      <sheetName val="Methods Overview"/>
-      <sheetName val="Scenario Inputs"/>
-      <sheetName val="Settings"/>
-      <sheetName val="Cost Inputs"/>
-      <sheetName val="References"/>
-      <sheetName val="simPy_sheet"/>
-      <sheetName val="age_dist_all_models"/>
-      <sheetName val="daily_rate_profiles_all_models"/>
-      <sheetName val="tw_tx_all_models"/>
-      <sheetName val="tw_tx"/>
-      <sheetName val="Inputs Graph Data"/>
-      <sheetName val="Hide Selection Settings"/>
-      <sheetName val="Model Interface"/>
-      <sheetName val="Model Indexing"/>
-      <sheetName val="Prev_Pop_Initialisation"/>
-      <sheetName val="Prev_Pop_all_models"/>
-      <sheetName val="prevalent_population"/>
-      <sheetName val="prevalent_population_all_models"/>
-      <sheetName val="age_dist"/>
-      <sheetName val="ethnicity_dist_all_models"/>
-      <sheetName val="referral_dist"/>
-      <sheetName val="referral_dist_all_models"/>
-      <sheetName val="daily_rate"/>
-      <sheetName val="CKD baseline inputs"/>
-      <sheetName val="divertToCC"/>
-      <sheetName val="suitableForTx"/>
-      <sheetName val="suitableForTx_all_models"/>
-      <sheetName val="preE_Tx_Cadav"/>
-      <sheetName val="preE_Tx_Cadav_all_models"/>
-      <sheetName val="preE_Tx_Live"/>
-      <sheetName val="preE_Tx_Live_all_models"/>
-      <sheetName val="modAllocation"/>
-      <sheetName val="modAllocation_all_models"/>
-      <sheetName val="TxType"/>
-      <sheetName val="TxType_all_models"/>
-      <sheetName val="receivesTx"/>
-      <sheetName val="receivesTx_all_models"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5">
-        <row r="51">
-          <cell r="I51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="J51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="K51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="L51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="M51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="N51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="O51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="P51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="Q51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="R51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="S51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="T51">
-            <v>0.14691943127962084</v>
-          </cell>
-          <cell r="U51">
-            <v>0.14691943127962084</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34"/>
-      <sheetData sheetId="35"/>
-      <sheetData sheetId="36"/>
-      <sheetData sheetId="37"/>
-      <sheetData sheetId="38"/>
-      <sheetData sheetId="39"/>
-      <sheetData sheetId="40"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Lucy Morgan (Strategy Unit, hosted by ML)" id="{1A249F06-EDDD-42AB-8413-B80F61FA87C3}" userId="S::Lucy.Morgan@mlcsu.nhs.uk::e5e54b71-cf62-4ad2-985a-344b32ab1816" providerId="AD"/>
@@ -26712,7 +26572,7 @@
       <c r="B1" s="4">
         <v>0.7</v>
       </c>
-      <c r="C1" s="181" t="s">
+      <c r="C1" s="183" t="s">
         <v>158</v>
       </c>
     </row>
@@ -26723,7 +26583,7 @@
       <c r="B2" s="4">
         <v>0.6</v>
       </c>
-      <c r="C2" s="181"/>
+      <c r="C2" s="183"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4">
@@ -26732,7 +26592,7 @@
       <c r="B3" s="4">
         <v>0.5</v>
       </c>
-      <c r="C3" s="181"/>
+      <c r="C3" s="183"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4">
@@ -26741,7 +26601,7 @@
       <c r="B4" s="4">
         <v>0.4</v>
       </c>
-      <c r="C4" s="181"/>
+      <c r="C4" s="183"/>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="4">
@@ -26750,7 +26610,7 @@
       <c r="B5" s="4">
         <v>0.2</v>
       </c>
-      <c r="C5" s="181"/>
+      <c r="C5" s="183"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="4">
@@ -26759,7 +26619,7 @@
       <c r="B6" s="4">
         <v>0.05</v>
       </c>
-      <c r="C6" s="181"/>
+      <c r="C6" s="183"/>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="4">
@@ -26768,7 +26628,7 @@
       <c r="B9" s="4">
         <v>0.7</v>
       </c>
-      <c r="C9" s="181" t="s">
+      <c r="C9" s="183" t="s">
         <v>157</v>
       </c>
     </row>
@@ -26779,7 +26639,7 @@
       <c r="B10" s="4">
         <v>0.6</v>
       </c>
-      <c r="C10" s="181"/>
+      <c r="C10" s="183"/>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="4">
@@ -26788,7 +26648,7 @@
       <c r="B11" s="4">
         <v>0.5</v>
       </c>
-      <c r="C11" s="181"/>
+      <c r="C11" s="183"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="4">
@@ -26797,7 +26657,7 @@
       <c r="B12" s="4">
         <v>0.4</v>
       </c>
-      <c r="C12" s="181"/>
+      <c r="C12" s="183"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="4">
@@ -26806,7 +26666,7 @@
       <c r="B13" s="4">
         <v>0.2</v>
       </c>
-      <c r="C13" s="181"/>
+      <c r="C13" s="183"/>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="4">
@@ -26815,7 +26675,7 @@
       <c r="B14" s="4">
         <v>0.05</v>
       </c>
-      <c r="C14" s="181"/>
+      <c r="C14" s="183"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -28218,21 +28078,21 @@
       <c r="C13" s="4"/>
     </row>
     <row r="14" spans="1:16" ht="16.95" hidden="1" customHeight="1">
-      <c r="B14" s="182" t="s">
+      <c r="B14" s="184" t="s">
         <v>85</v>
       </c>
-      <c r="C14" s="182"/>
-      <c r="D14" s="182"/>
-      <c r="E14" s="182"/>
-      <c r="F14" s="182"/>
-      <c r="G14" s="182"/>
-      <c r="H14" s="182"/>
-      <c r="I14" s="182"/>
-      <c r="J14" s="182"/>
-      <c r="K14" s="182"/>
-      <c r="L14" s="182"/>
-      <c r="M14" s="182"/>
-      <c r="N14" s="182"/>
+      <c r="C14" s="184"/>
+      <c r="D14" s="184"/>
+      <c r="E14" s="184"/>
+      <c r="F14" s="184"/>
+      <c r="G14" s="184"/>
+      <c r="H14" s="184"/>
+      <c r="I14" s="184"/>
+      <c r="J14" s="184"/>
+      <c r="K14" s="184"/>
+      <c r="L14" s="184"/>
+      <c r="M14" s="184"/>
+      <c r="N14" s="184"/>
     </row>
     <row r="15" spans="1:16" hidden="1">
       <c r="B15">
@@ -28394,21 +28254,21 @@
     </row>
     <row r="19" spans="1:15" ht="15">
       <c r="A19" s="13"/>
-      <c r="B19" s="182" t="s">
+      <c r="B19" s="184" t="s">
         <v>85</v>
       </c>
-      <c r="C19" s="182"/>
-      <c r="D19" s="182"/>
-      <c r="E19" s="182"/>
-      <c r="F19" s="182"/>
-      <c r="G19" s="182"/>
-      <c r="H19" s="182"/>
-      <c r="I19" s="182"/>
-      <c r="J19" s="182"/>
-      <c r="K19" s="182"/>
-      <c r="L19" s="182"/>
-      <c r="M19" s="182"/>
-      <c r="N19" s="182"/>
+      <c r="C19" s="184"/>
+      <c r="D19" s="184"/>
+      <c r="E19" s="184"/>
+      <c r="F19" s="184"/>
+      <c r="G19" s="184"/>
+      <c r="H19" s="184"/>
+      <c r="I19" s="184"/>
+      <c r="J19" s="184"/>
+      <c r="K19" s="184"/>
+      <c r="L19" s="184"/>
+      <c r="M19" s="184"/>
+      <c r="N19" s="184"/>
     </row>
     <row r="20" spans="1:15">
       <c r="B20">
@@ -29247,36 +29107,36 @@
       </c>
     </row>
     <row r="45" spans="1:28" hidden="1">
-      <c r="C45" s="182" t="s">
+      <c r="C45" s="184" t="s">
         <v>61</v>
       </c>
-      <c r="D45" s="182"/>
-      <c r="E45" s="182"/>
-      <c r="F45" s="182"/>
-      <c r="G45" s="182"/>
-      <c r="H45" s="182"/>
-      <c r="I45" s="182"/>
-      <c r="J45" s="182"/>
-      <c r="K45" s="182"/>
-      <c r="L45" s="182"/>
-      <c r="M45" s="182"/>
-      <c r="N45" s="182"/>
-      <c r="O45" s="182"/>
-      <c r="P45" s="182" t="s">
+      <c r="D45" s="184"/>
+      <c r="E45" s="184"/>
+      <c r="F45" s="184"/>
+      <c r="G45" s="184"/>
+      <c r="H45" s="184"/>
+      <c r="I45" s="184"/>
+      <c r="J45" s="184"/>
+      <c r="K45" s="184"/>
+      <c r="L45" s="184"/>
+      <c r="M45" s="184"/>
+      <c r="N45" s="184"/>
+      <c r="O45" s="184"/>
+      <c r="P45" s="184" t="s">
         <v>132</v>
       </c>
-      <c r="Q45" s="182"/>
-      <c r="R45" s="182"/>
-      <c r="S45" s="182"/>
-      <c r="T45" s="182"/>
-      <c r="U45" s="182"/>
-      <c r="V45" s="182"/>
-      <c r="W45" s="182"/>
-      <c r="X45" s="182"/>
-      <c r="Y45" s="182"/>
-      <c r="Z45" s="182"/>
-      <c r="AA45" s="182"/>
-      <c r="AB45" s="182"/>
+      <c r="Q45" s="184"/>
+      <c r="R45" s="184"/>
+      <c r="S45" s="184"/>
+      <c r="T45" s="184"/>
+      <c r="U45" s="184"/>
+      <c r="V45" s="184"/>
+      <c r="W45" s="184"/>
+      <c r="X45" s="184"/>
+      <c r="Y45" s="184"/>
+      <c r="Z45" s="184"/>
+      <c r="AA45" s="184"/>
+      <c r="AB45" s="184"/>
     </row>
     <row r="46" spans="1:28" ht="19.2">
       <c r="A46" s="44" t="s">
@@ -33971,11 +33831,11 @@
         <v>109</v>
       </c>
       <c r="B104" s="4"/>
-      <c r="C104" s="181" t="s">
+      <c r="C104" s="183" t="s">
         <v>157</v>
       </c>
-      <c r="D104" s="181"/>
-      <c r="E104" s="181"/>
+      <c r="D104" s="183"/>
+      <c r="E104" s="183"/>
       <c r="G104" t="s">
         <v>158</v>
       </c>
@@ -36062,57 +35922,57 @@
         <f>G169/SUM(G155,G169,G183)</f>
         <v>0.1891891891891892</v>
       </c>
-      <c r="C255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!I49="","",'[1]Scenario Inputs'!I51)</f>
-        <v/>
-      </c>
-      <c r="D255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!J49="","",'[1]Scenario Inputs'!J51)</f>
-        <v/>
-      </c>
-      <c r="E255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!K49="","",'[1]Scenario Inputs'!K51)</f>
-        <v/>
-      </c>
-      <c r="F255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!L49="","",'[1]Scenario Inputs'!L51)</f>
-        <v/>
-      </c>
-      <c r="G255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!M49="","",'[1]Scenario Inputs'!M51)</f>
-        <v/>
-      </c>
-      <c r="H255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!N49="","",'[1]Scenario Inputs'!N51)</f>
-        <v/>
-      </c>
-      <c r="I255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!O49="","",'[1]Scenario Inputs'!O51)</f>
-        <v/>
-      </c>
-      <c r="J255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!P49="","",'[1]Scenario Inputs'!P51)</f>
-        <v/>
-      </c>
-      <c r="K255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!Q49="","",'[1]Scenario Inputs'!Q51)</f>
-        <v/>
-      </c>
-      <c r="L255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!R49="","",'[1]Scenario Inputs'!R51)</f>
-        <v/>
-      </c>
-      <c r="M255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!S49="","",'[1]Scenario Inputs'!S51)</f>
-        <v/>
-      </c>
-      <c r="N255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!T49="","",'[1]Scenario Inputs'!T51)</f>
-        <v/>
-      </c>
-      <c r="O255" s="2" t="str">
-        <f>IF('[1]Scenario Inputs'!U49="","",'[1]Scenario Inputs'!U51)</f>
-        <v/>
+      <c r="C255" s="2">
+        <f>IF('Scenario Inputs'!I49="",-1,'Scenario Inputs'!I51)</f>
+        <v>-1</v>
+      </c>
+      <c r="D255" s="2">
+        <f>IF('Scenario Inputs'!J49="",-1,'Scenario Inputs'!J51)</f>
+        <v>-1</v>
+      </c>
+      <c r="E255" s="2">
+        <f>IF('Scenario Inputs'!K49="",-1,'Scenario Inputs'!K51)</f>
+        <v>-1</v>
+      </c>
+      <c r="F255" s="2">
+        <f>IF('Scenario Inputs'!L49="",-1,'Scenario Inputs'!L51)</f>
+        <v>-1</v>
+      </c>
+      <c r="G255" s="2">
+        <f>IF('Scenario Inputs'!M49="",-1,'Scenario Inputs'!M51)</f>
+        <v>-1</v>
+      </c>
+      <c r="H255" s="2">
+        <f>IF('Scenario Inputs'!N49="",-1,'Scenario Inputs'!N51)</f>
+        <v>-1</v>
+      </c>
+      <c r="I255" s="2">
+        <f>IF('Scenario Inputs'!O49="",-1,'Scenario Inputs'!O51)</f>
+        <v>-1</v>
+      </c>
+      <c r="J255" s="2">
+        <f>IF('Scenario Inputs'!P49="",-1,'Scenario Inputs'!P51)</f>
+        <v>-1</v>
+      </c>
+      <c r="K255" s="2">
+        <f>IF('Scenario Inputs'!Q49="",-1,'Scenario Inputs'!Q51)</f>
+        <v>-1</v>
+      </c>
+      <c r="L255" s="2">
+        <f>IF('Scenario Inputs'!R49="",-1,'Scenario Inputs'!R51)</f>
+        <v>-1</v>
+      </c>
+      <c r="M255" s="2">
+        <f>IF('Scenario Inputs'!S49="",-1,'Scenario Inputs'!S51)</f>
+        <v>-1</v>
+      </c>
+      <c r="N255" s="2">
+        <f>IF('Scenario Inputs'!T49="",-1,'Scenario Inputs'!T51)</f>
+        <v>-1</v>
+      </c>
+      <c r="O255" s="2">
+        <f>IF('Scenario Inputs'!U49="",-1,'Scenario Inputs'!U51)</f>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>
@@ -36235,15 +36095,15 @@
       <c r="C18" s="131" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="157"/>
-      <c r="E18" s="157"/>
-      <c r="F18" s="157"/>
-      <c r="G18" s="157"/>
-      <c r="H18" s="157"/>
-      <c r="I18" s="157"/>
-      <c r="J18" s="157"/>
-      <c r="K18" s="157"/>
-      <c r="L18" s="157"/>
+      <c r="D18" s="142"/>
+      <c r="E18" s="142"/>
+      <c r="F18" s="142"/>
+      <c r="G18" s="142"/>
+      <c r="H18" s="142"/>
+      <c r="I18" s="142"/>
+      <c r="J18" s="142"/>
+      <c r="K18" s="142"/>
+      <c r="L18" s="142"/>
       <c r="M18" s="125"/>
       <c r="N18" s="131" t="s">
         <v>71</v>
@@ -36289,27 +36149,27 @@
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
-      <c r="F20" s="151" t="s">
+      <c r="F20" s="143" t="s">
         <v>177</v>
       </c>
-      <c r="G20" s="151"/>
-      <c r="H20" s="151"/>
-      <c r="I20" s="151"/>
-      <c r="J20" s="151"/>
-      <c r="K20" s="151"/>
-      <c r="L20" s="151"/>
+      <c r="G20" s="143"/>
+      <c r="H20" s="143"/>
+      <c r="I20" s="143"/>
+      <c r="J20" s="143"/>
+      <c r="K20" s="143"/>
+      <c r="L20" s="143"/>
       <c r="M20" s="6"/>
       <c r="N20" s="11"/>
       <c r="O20" s="11"/>
       <c r="P20" s="11"/>
       <c r="Q20" s="11"/>
-      <c r="R20" s="158"/>
-      <c r="S20" s="158"/>
-      <c r="T20" s="158"/>
-      <c r="U20" s="158"/>
-      <c r="V20" s="158"/>
-      <c r="W20" s="158"/>
-      <c r="X20" s="158"/>
+      <c r="R20" s="144"/>
+      <c r="S20" s="144"/>
+      <c r="T20" s="144"/>
+      <c r="U20" s="144"/>
+      <c r="V20" s="144"/>
+      <c r="W20" s="144"/>
+      <c r="X20" s="144"/>
     </row>
     <row r="21" spans="3:24" ht="16.8">
       <c r="C21" s="6" t="s">
@@ -36317,15 +36177,15 @@
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
-      <c r="F21" s="151" t="s">
+      <c r="F21" s="143" t="s">
         <v>178</v>
       </c>
-      <c r="G21" s="151"/>
-      <c r="H21" s="151"/>
-      <c r="I21" s="151"/>
-      <c r="J21" s="151"/>
-      <c r="K21" s="151"/>
-      <c r="L21" s="151"/>
+      <c r="G21" s="143"/>
+      <c r="H21" s="143"/>
+      <c r="I21" s="143"/>
+      <c r="J21" s="143"/>
+      <c r="K21" s="143"/>
+      <c r="L21" s="143"/>
       <c r="M21" s="6"/>
       <c r="N21" s="6" t="s">
         <v>6</v>
@@ -36333,15 +36193,15 @@
       <c r="O21" s="6"/>
       <c r="P21" s="6"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="159">
+      <c r="R21" s="145">
         <v>2023</v>
       </c>
-      <c r="S21" s="160"/>
-      <c r="T21" s="160"/>
-      <c r="U21" s="160"/>
-      <c r="V21" s="160"/>
-      <c r="W21" s="160"/>
-      <c r="X21" s="161"/>
+      <c r="S21" s="146"/>
+      <c r="T21" s="146"/>
+      <c r="U21" s="146"/>
+      <c r="V21" s="146"/>
+      <c r="W21" s="146"/>
+      <c r="X21" s="147"/>
     </row>
     <row r="22" spans="3:24" ht="16.95" hidden="1" customHeight="1">
       <c r="C22" s="6" t="s">
@@ -36349,15 +36209,15 @@
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
-      <c r="F22" s="151" t="s">
+      <c r="F22" s="143" t="s">
         <v>8</v>
       </c>
-      <c r="G22" s="151"/>
-      <c r="H22" s="151"/>
-      <c r="I22" s="151"/>
-      <c r="J22" s="151"/>
-      <c r="K22" s="151"/>
-      <c r="L22" s="151"/>
+      <c r="G22" s="143"/>
+      <c r="H22" s="143"/>
+      <c r="I22" s="143"/>
+      <c r="J22" s="143"/>
+      <c r="K22" s="143"/>
+      <c r="L22" s="143"/>
       <c r="M22" s="6"/>
     </row>
     <row r="23" spans="3:24" ht="16.8">
@@ -36366,15 +36226,15 @@
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="151" t="s">
+      <c r="F23" s="143" t="s">
         <v>22</v>
       </c>
-      <c r="G23" s="151"/>
-      <c r="H23" s="151"/>
-      <c r="I23" s="151"/>
-      <c r="J23" s="151"/>
-      <c r="K23" s="151"/>
-      <c r="L23" s="151"/>
+      <c r="G23" s="143"/>
+      <c r="H23" s="143"/>
+      <c r="I23" s="143"/>
+      <c r="J23" s="143"/>
+      <c r="K23" s="143"/>
+      <c r="L23" s="143"/>
       <c r="M23" s="6"/>
       <c r="N23" s="6" t="s">
         <v>11</v>
@@ -36382,15 +36242,15 @@
       <c r="O23" s="6"/>
       <c r="P23" s="6"/>
       <c r="Q23" s="6"/>
-      <c r="R23" s="152">
+      <c r="R23" s="148">
         <v>2035</v>
       </c>
-      <c r="S23" s="153"/>
-      <c r="T23" s="153"/>
-      <c r="U23" s="153"/>
-      <c r="V23" s="153"/>
-      <c r="W23" s="153"/>
-      <c r="X23" s="154"/>
+      <c r="S23" s="149"/>
+      <c r="T23" s="149"/>
+      <c r="U23" s="149"/>
+      <c r="V23" s="149"/>
+      <c r="W23" s="149"/>
+      <c r="X23" s="150"/>
     </row>
     <row r="24" spans="3:24" ht="16.8">
       <c r="C24" s="110"/>
@@ -36435,15 +36295,15 @@
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="8"/>
-      <c r="T25" s="149" t="s">
+      <c r="T25" s="151" t="s">
         <v>13</v>
       </c>
-      <c r="U25" s="149"/>
-      <c r="V25" s="155" t="s">
+      <c r="U25" s="151"/>
+      <c r="V25" s="152" t="s">
         <v>14</v>
       </c>
-      <c r="W25" s="156"/>
-      <c r="X25" s="156"/>
+      <c r="W25" s="153"/>
+      <c r="X25" s="153"/>
     </row>
     <row r="26" spans="3:24" ht="16.95" hidden="1" customHeight="1">
       <c r="C26" s="6"/>
@@ -36464,17 +36324,17 @@
       <c r="P26" s="6"/>
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
-      <c r="T26" s="163">
+      <c r="T26" s="132">
         <f>G49</f>
         <v>0.1891891891891892</v>
       </c>
-      <c r="U26" s="164"/>
-      <c r="V26" s="165">
+      <c r="U26" s="133"/>
+      <c r="V26" s="134">
         <f>K49</f>
         <v>0</v>
       </c>
-      <c r="W26" s="166"/>
-      <c r="X26" s="167"/>
+      <c r="W26" s="135"/>
+      <c r="X26" s="136"/>
     </row>
     <row r="27" spans="3:24" ht="16.95" hidden="1" customHeight="1">
       <c r="C27" s="6"/>
@@ -36496,17 +36356,17 @@
       <c r="P27" s="6"/>
       <c r="Q27" s="6"/>
       <c r="R27" s="6"/>
-      <c r="T27" s="163">
+      <c r="T27" s="132">
         <f>G52</f>
         <v>0.28999999999999998</v>
       </c>
-      <c r="U27" s="164"/>
-      <c r="V27" s="165">
+      <c r="U27" s="133"/>
+      <c r="V27" s="134">
         <f>K52</f>
         <v>0</v>
       </c>
-      <c r="W27" s="166"/>
-      <c r="X27" s="167"/>
+      <c r="W27" s="135"/>
+      <c r="X27" s="136"/>
     </row>
     <row r="28" spans="3:24" ht="16.95" hidden="1" customHeight="1">
       <c r="C28" s="6"/>
@@ -36528,17 +36388,17 @@
       <c r="P28" s="6"/>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
-      <c r="T28" s="163" t="e">
+      <c r="T28" s="132" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="U28" s="164"/>
-      <c r="V28" s="165" t="e">
+      <c r="U28" s="133"/>
+      <c r="V28" s="134" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="W28" s="166"/>
-      <c r="X28" s="167"/>
+      <c r="W28" s="135"/>
+      <c r="X28" s="136"/>
     </row>
     <row r="29" spans="3:24" ht="16.95" hidden="1" customHeight="1">
       <c r="C29" s="6"/>
@@ -36560,17 +36420,17 @@
       <c r="P29" s="6"/>
       <c r="Q29" s="6"/>
       <c r="R29" s="6"/>
-      <c r="T29" s="163" t="e">
+      <c r="T29" s="132" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="U29" s="164"/>
-      <c r="V29" s="165" t="e">
+      <c r="U29" s="133"/>
+      <c r="V29" s="134" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="W29" s="166"/>
-      <c r="X29" s="167"/>
+      <c r="W29" s="135"/>
+      <c r="X29" s="136"/>
     </row>
     <row r="30" spans="3:24" ht="16.95" hidden="1" customHeight="1">
       <c r="C30" s="6"/>
@@ -36592,17 +36452,17 @@
       <c r="P30" s="6"/>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
-      <c r="T30" s="163">
+      <c r="T30" s="132">
         <f>G75</f>
         <v>0.9</v>
       </c>
-      <c r="U30" s="164"/>
-      <c r="V30" s="165">
+      <c r="U30" s="133"/>
+      <c r="V30" s="134">
         <f>K75</f>
         <v>0</v>
       </c>
-      <c r="W30" s="166"/>
-      <c r="X30" s="167"/>
+      <c r="W30" s="135"/>
+      <c r="X30" s="136"/>
     </row>
     <row r="31" spans="3:24" ht="16.95" hidden="1" customHeight="1">
       <c r="C31" s="6"/>
@@ -36624,17 +36484,17 @@
       <c r="P31" s="6"/>
       <c r="Q31" s="6"/>
       <c r="R31" s="6"/>
-      <c r="T31" s="168">
+      <c r="T31" s="137">
         <f>G78</f>
         <v>0.5</v>
       </c>
-      <c r="U31" s="169"/>
-      <c r="V31" s="170">
+      <c r="U31" s="138"/>
+      <c r="V31" s="139">
         <f>K78</f>
         <v>0</v>
       </c>
-      <c r="W31" s="171"/>
-      <c r="X31" s="172"/>
+      <c r="W31" s="140"/>
+      <c r="X31" s="141"/>
     </row>
     <row r="32" spans="3:24" ht="16.8" hidden="1">
       <c r="C32" s="6"/>
@@ -36738,25 +36598,25 @@
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
-      <c r="G36" s="143" t="s">
+      <c r="G36" s="156" t="s">
         <v>134</v>
       </c>
-      <c r="H36" s="143"/>
-      <c r="I36" s="149" t="s">
+      <c r="H36" s="156"/>
+      <c r="I36" s="151" t="s">
         <v>56</v>
       </c>
-      <c r="J36" s="149"/>
-      <c r="K36" s="149"/>
-      <c r="L36" s="149"/>
-      <c r="M36" s="149"/>
-      <c r="N36" s="149"/>
-      <c r="O36" s="149"/>
-      <c r="P36" s="149"/>
-      <c r="Q36" s="149"/>
-      <c r="R36" s="149"/>
-      <c r="S36" s="149"/>
-      <c r="T36" s="149"/>
-      <c r="U36" s="149"/>
+      <c r="J36" s="151"/>
+      <c r="K36" s="151"/>
+      <c r="L36" s="151"/>
+      <c r="M36" s="151"/>
+      <c r="N36" s="151"/>
+      <c r="O36" s="151"/>
+      <c r="P36" s="151"/>
+      <c r="Q36" s="151"/>
+      <c r="R36" s="151"/>
+      <c r="S36" s="151"/>
+      <c r="T36" s="151"/>
+      <c r="U36" s="151"/>
       <c r="V36" s="118"/>
       <c r="W36" s="118"/>
       <c r="X36" s="118"/>
@@ -36766,8 +36626,8 @@
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
-      <c r="G37" s="144"/>
-      <c r="H37" s="144"/>
+      <c r="G37" s="157"/>
+      <c r="H37" s="157"/>
       <c r="I37" s="119">
         <v>2023</v>
       </c>
@@ -36818,10 +36678,10 @@
       <c r="D38" s="12"/>
       <c r="E38" s="12"/>
       <c r="F38" s="12"/>
-      <c r="G38" s="147">
+      <c r="G38" s="154">
         <v>1</v>
       </c>
-      <c r="H38" s="148"/>
+      <c r="H38" s="155"/>
       <c r="I38" s="121"/>
       <c r="J38" s="121"/>
       <c r="K38" s="121"/>
@@ -36844,10 +36704,10 @@
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
-      <c r="G39" s="150" t="s">
+      <c r="G39" s="158" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="150"/>
+      <c r="H39" s="158"/>
       <c r="I39" s="122">
         <f>daily_rate!N2</f>
         <v>0.5</v>
@@ -36909,10 +36769,10 @@
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
-      <c r="G40" s="135" t="s">
+      <c r="G40" s="171" t="s">
         <v>182</v>
       </c>
-      <c r="H40" s="135"/>
+      <c r="H40" s="171"/>
       <c r="I40" s="123">
         <f>simPy_sheet!B6</f>
         <v>0.5</v>
@@ -37120,25 +36980,25 @@
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
-      <c r="G47" s="143" t="s">
+      <c r="G47" s="156" t="s">
         <v>17</v>
       </c>
-      <c r="H47" s="143"/>
-      <c r="I47" s="132" t="s">
+      <c r="H47" s="156"/>
+      <c r="I47" s="167" t="s">
         <v>85</v>
       </c>
-      <c r="J47" s="133"/>
-      <c r="K47" s="133"/>
-      <c r="L47" s="133"/>
-      <c r="M47" s="133"/>
-      <c r="N47" s="133"/>
-      <c r="O47" s="133"/>
-      <c r="P47" s="133"/>
-      <c r="Q47" s="133"/>
-      <c r="R47" s="133"/>
-      <c r="S47" s="133"/>
-      <c r="T47" s="133"/>
-      <c r="U47" s="134"/>
+      <c r="J47" s="168"/>
+      <c r="K47" s="168"/>
+      <c r="L47" s="168"/>
+      <c r="M47" s="168"/>
+      <c r="N47" s="168"/>
+      <c r="O47" s="168"/>
+      <c r="P47" s="168"/>
+      <c r="Q47" s="168"/>
+      <c r="R47" s="168"/>
+      <c r="S47" s="168"/>
+      <c r="T47" s="168"/>
+      <c r="U47" s="169"/>
       <c r="V47" s="6"/>
       <c r="W47" s="6"/>
       <c r="X47" s="6"/>
@@ -37160,8 +37020,8 @@
       <c r="D48" s="15"/>
       <c r="E48" s="15"/>
       <c r="F48" s="15"/>
-      <c r="G48" s="144"/>
-      <c r="H48" s="144"/>
+      <c r="G48" s="157"/>
+      <c r="H48" s="157"/>
       <c r="I48">
         <f>R21</f>
         <v>2023</v>
@@ -37237,11 +37097,11 @@
       <c r="D49" s="12"/>
       <c r="E49" s="12"/>
       <c r="F49" s="109"/>
-      <c r="G49" s="226">
+      <c r="G49" s="178">
         <f>simPy_sheet!B255</f>
         <v>0.1891891891891892</v>
       </c>
-      <c r="H49" s="227"/>
+      <c r="H49" s="179"/>
       <c r="I49" s="68"/>
       <c r="J49" s="68"/>
       <c r="K49" s="68"/>
@@ -37264,10 +37124,10 @@
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
-      <c r="G50" s="162" t="s">
+      <c r="G50" s="177" t="s">
         <v>183</v>
       </c>
-      <c r="H50" s="162"/>
+      <c r="H50" s="177"/>
       <c r="I50" s="108">
         <f t="shared" ref="I50:U50" si="1">IncHHD</f>
         <v>0.1891891891891892</v>
@@ -37329,10 +37189,10 @@
       <c r="D51" s="6"/>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
-      <c r="G51" s="162" t="s">
+      <c r="G51" s="177" t="s">
         <v>184</v>
       </c>
-      <c r="H51" s="162"/>
+      <c r="H51" s="177"/>
       <c r="I51" s="108">
         <f>AVERAGE(simPy_sheet!G77:G82)</f>
         <v>0.18918918918918923</v>
@@ -37396,11 +37256,11 @@
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
       <c r="F52" s="103"/>
-      <c r="G52" s="129">
+      <c r="G52" s="180">
         <f>modAllocation!E1</f>
         <v>0.28999999999999998</v>
       </c>
-      <c r="H52" s="130"/>
+      <c r="H52" s="181"/>
       <c r="I52" s="68"/>
       <c r="J52" s="68"/>
       <c r="K52" s="68"/>
@@ -37423,10 +37283,10 @@
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
-      <c r="G53" s="176" t="s">
+      <c r="G53" s="182" t="s">
         <v>183</v>
       </c>
-      <c r="H53" s="176"/>
+      <c r="H53" s="182"/>
       <c r="I53" s="90">
         <f>AVERAGE(simPy_sheet!$E$71:$E$76)</f>
         <v>0.28999999999999998</v>
@@ -37488,10 +37348,10 @@
       <c r="D54" s="6"/>
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
-      <c r="G54" s="135" t="s">
+      <c r="G54" s="171" t="s">
         <v>184</v>
       </c>
-      <c r="H54" s="135"/>
+      <c r="H54" s="171"/>
       <c r="I54" s="90">
         <f>AVERAGE(simPy_sheet!H71:H76)</f>
         <v>0.28999999999999998</v>
@@ -37653,25 +37513,25 @@
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
       <c r="F59" s="6"/>
-      <c r="G59" s="143" t="s">
+      <c r="G59" s="156" t="s">
         <v>17</v>
       </c>
-      <c r="H59" s="143"/>
-      <c r="I59" s="132" t="s">
+      <c r="H59" s="156"/>
+      <c r="I59" s="167" t="s">
         <v>85</v>
       </c>
-      <c r="J59" s="133"/>
-      <c r="K59" s="133"/>
-      <c r="L59" s="133"/>
-      <c r="M59" s="133"/>
-      <c r="N59" s="133"/>
-      <c r="O59" s="133"/>
-      <c r="P59" s="133"/>
-      <c r="Q59" s="133"/>
-      <c r="R59" s="133"/>
-      <c r="S59" s="133"/>
-      <c r="T59" s="133"/>
-      <c r="U59" s="134"/>
+      <c r="J59" s="168"/>
+      <c r="K59" s="168"/>
+      <c r="L59" s="168"/>
+      <c r="M59" s="168"/>
+      <c r="N59" s="168"/>
+      <c r="O59" s="168"/>
+      <c r="P59" s="168"/>
+      <c r="Q59" s="168"/>
+      <c r="R59" s="168"/>
+      <c r="S59" s="168"/>
+      <c r="T59" s="168"/>
+      <c r="U59" s="169"/>
       <c r="V59" s="6"/>
       <c r="W59" s="6"/>
       <c r="X59" s="6"/>
@@ -37683,8 +37543,8 @@
       <c r="F60" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G60" s="144"/>
-      <c r="H60" s="144"/>
+      <c r="G60" s="157"/>
+      <c r="H60" s="157"/>
       <c r="I60">
         <f>R21</f>
         <v>2023</v>
@@ -37750,11 +37610,11 @@
       <c r="F61" s="97" t="s">
         <v>87</v>
       </c>
-      <c r="G61" s="137">
+      <c r="G61" s="159">
         <f>divertToCC!C1</f>
         <v>0.1</v>
       </c>
-      <c r="H61" s="138"/>
+      <c r="H61" s="160"/>
       <c r="I61" s="68"/>
       <c r="J61" s="68"/>
       <c r="K61" s="68"/>
@@ -37779,11 +37639,11 @@
       <c r="F62" s="98" t="s">
         <v>88</v>
       </c>
-      <c r="G62" s="137">
+      <c r="G62" s="159">
         <f>divertToCC!C2</f>
         <v>0.1</v>
       </c>
-      <c r="H62" s="138"/>
+      <c r="H62" s="160"/>
       <c r="I62" s="68"/>
       <c r="J62" s="68"/>
       <c r="K62" s="68"/>
@@ -37808,11 +37668,11 @@
       <c r="F63" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="G63" s="137">
+      <c r="G63" s="159">
         <f>divertToCC!C3</f>
         <v>0.1</v>
       </c>
-      <c r="H63" s="138"/>
+      <c r="H63" s="160"/>
       <c r="I63" s="68"/>
       <c r="J63" s="68"/>
       <c r="K63" s="68"/>
@@ -37837,11 +37697,11 @@
       <c r="F64" s="98" t="s">
         <v>90</v>
       </c>
-      <c r="G64" s="137">
+      <c r="G64" s="159">
         <f>divertToCC!C4</f>
         <v>0.1</v>
       </c>
-      <c r="H64" s="138"/>
+      <c r="H64" s="160"/>
       <c r="I64" s="68"/>
       <c r="J64" s="68"/>
       <c r="K64" s="68"/>
@@ -37866,11 +37726,11 @@
       <c r="F65" s="98" t="s">
         <v>91</v>
       </c>
-      <c r="G65" s="137">
+      <c r="G65" s="159">
         <f>divertToCC!C5</f>
         <v>0.25</v>
       </c>
-      <c r="H65" s="138"/>
+      <c r="H65" s="160"/>
       <c r="I65" s="68"/>
       <c r="J65" s="68"/>
       <c r="K65" s="68"/>
@@ -37895,11 +37755,11 @@
       <c r="F66" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="G66" s="139">
+      <c r="G66" s="164">
         <f>divertToCC!C6</f>
         <v>0.5</v>
       </c>
-      <c r="H66" s="140"/>
+      <c r="H66" s="165"/>
       <c r="I66" s="69"/>
       <c r="J66" s="69"/>
       <c r="K66" s="69"/>
@@ -37924,11 +37784,11 @@
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
       <c r="F67" s="103"/>
-      <c r="G67" s="145">
+      <c r="G67" s="161">
         <f>referral_dist!B2</f>
         <v>0.2</v>
       </c>
-      <c r="H67" s="146"/>
+      <c r="H67" s="162"/>
       <c r="I67" s="70"/>
       <c r="J67" s="70"/>
       <c r="K67" s="70"/>
@@ -37951,10 +37811,10 @@
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
       <c r="F68" s="6"/>
-      <c r="G68" s="142" t="s">
+      <c r="G68" s="170" t="s">
         <v>185</v>
       </c>
-      <c r="H68" s="142"/>
+      <c r="H68" s="170"/>
       <c r="I68" s="100">
         <f t="shared" ref="I68:U68" si="3">IncLP</f>
         <v>0.2</v>
@@ -38016,10 +37876,10 @@
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
-      <c r="G69" s="135" t="s">
+      <c r="G69" s="171" t="s">
         <v>186</v>
       </c>
-      <c r="H69" s="135"/>
+      <c r="H69" s="171"/>
       <c r="I69" s="101">
         <f>simPy_sheet!B12</f>
         <v>0.2</v>
@@ -38150,21 +38010,21 @@
       <c r="F73" s="11"/>
       <c r="G73" s="11"/>
       <c r="H73" s="11"/>
-      <c r="I73" s="132" t="s">
+      <c r="I73" s="167" t="s">
         <v>137</v>
       </c>
-      <c r="J73" s="133"/>
-      <c r="K73" s="133"/>
-      <c r="L73" s="133"/>
-      <c r="M73" s="133"/>
-      <c r="N73" s="133"/>
-      <c r="O73" s="133"/>
-      <c r="P73" s="133"/>
-      <c r="Q73" s="133"/>
-      <c r="R73" s="133"/>
-      <c r="S73" s="133"/>
-      <c r="T73" s="133"/>
-      <c r="U73" s="134"/>
+      <c r="J73" s="168"/>
+      <c r="K73" s="168"/>
+      <c r="L73" s="168"/>
+      <c r="M73" s="168"/>
+      <c r="N73" s="168"/>
+      <c r="O73" s="168"/>
+      <c r="P73" s="168"/>
+      <c r="Q73" s="168"/>
+      <c r="R73" s="168"/>
+      <c r="S73" s="168"/>
+      <c r="T73" s="168"/>
+      <c r="U73" s="169"/>
     </row>
     <row r="74" spans="3:24" s="13" customFormat="1" ht="16.8" customHeight="1">
       <c r="C74" s="11"/>
@@ -38173,10 +38033,10 @@
       <c r="F74" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G74" s="174" t="s">
+      <c r="G74" s="173" t="s">
         <v>17</v>
       </c>
-      <c r="H74" s="174"/>
+      <c r="H74" s="173"/>
       <c r="I74">
         <f>R21</f>
         <v>2023</v>
@@ -38239,11 +38099,11 @@
       <c r="F75" s="97" t="s">
         <v>87</v>
       </c>
-      <c r="G75" s="175">
+      <c r="G75" s="129">
         <f>receivesTx!B1</f>
         <v>0.9</v>
       </c>
-      <c r="H75" s="175"/>
+      <c r="H75" s="129"/>
       <c r="I75" s="68"/>
       <c r="J75" s="68"/>
       <c r="K75" s="68"/>
@@ -38265,11 +38125,11 @@
       <c r="F76" s="98" t="s">
         <v>88</v>
       </c>
-      <c r="G76" s="175">
+      <c r="G76" s="129">
         <f>receivesTx!B2</f>
         <v>0.8</v>
       </c>
-      <c r="H76" s="175"/>
+      <c r="H76" s="129"/>
       <c r="I76" s="68"/>
       <c r="J76" s="68"/>
       <c r="K76" s="68"/>
@@ -38291,11 +38151,11 @@
       <c r="F77" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="G77" s="175">
+      <c r="G77" s="129">
         <f>receivesTx!B3</f>
         <v>0.6</v>
       </c>
-      <c r="H77" s="175"/>
+      <c r="H77" s="129"/>
       <c r="I77" s="68"/>
       <c r="J77" s="68"/>
       <c r="K77" s="68"/>
@@ -38317,11 +38177,11 @@
       <c r="F78" s="98" t="s">
         <v>90</v>
       </c>
-      <c r="G78" s="175">
+      <c r="G78" s="129">
         <f>receivesTx!B4</f>
         <v>0.5</v>
       </c>
-      <c r="H78" s="175"/>
+      <c r="H78" s="129"/>
       <c r="I78" s="68"/>
       <c r="J78" s="68"/>
       <c r="K78" s="68"/>
@@ -38343,11 +38203,11 @@
       <c r="F79" s="98" t="s">
         <v>91</v>
       </c>
-      <c r="G79" s="175">
+      <c r="G79" s="129">
         <f>receivesTx!B5</f>
         <v>0.5</v>
       </c>
-      <c r="H79" s="175"/>
+      <c r="H79" s="129"/>
       <c r="I79" s="68"/>
       <c r="J79" s="68"/>
       <c r="K79" s="68"/>
@@ -38369,11 +38229,11 @@
       <c r="F80" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="G80" s="180">
+      <c r="G80" s="130">
         <f>receivesTx!B6</f>
         <v>0</v>
       </c>
-      <c r="H80" s="180"/>
+      <c r="H80" s="130"/>
       <c r="I80" s="69"/>
       <c r="J80" s="69"/>
       <c r="K80" s="69"/>
@@ -38393,8 +38253,8 @@
       <c r="D81" s="11"/>
       <c r="E81" s="11"/>
       <c r="F81" s="11"/>
-      <c r="G81" s="141"/>
-      <c r="H81" s="141"/>
+      <c r="G81" s="166"/>
+      <c r="H81" s="166"/>
       <c r="I81" s="71"/>
       <c r="J81" s="71"/>
       <c r="K81" s="71"/>
@@ -38444,11 +38304,11 @@
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
       <c r="F83" s="88"/>
-      <c r="G83" s="177">
+      <c r="G83" s="174">
         <f>AVERAGE(simPy_sheet!AI57:AI62)</f>
         <v>0.19999999999999998</v>
       </c>
-      <c r="H83" s="178"/>
+      <c r="H83" s="175"/>
       <c r="I83" s="76"/>
       <c r="J83" s="76"/>
       <c r="K83" s="76"/>
@@ -38468,10 +38328,10 @@
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
       <c r="F84" s="88"/>
-      <c r="G84" s="179" t="s">
+      <c r="G84" s="176" t="s">
         <v>190</v>
       </c>
-      <c r="H84" s="179"/>
+      <c r="H84" s="176"/>
       <c r="I84" s="89">
         <f>$G$83</f>
         <v>0.19999999999999998</v>
@@ -38529,10 +38389,10 @@
       <c r="D85" s="11"/>
       <c r="E85" s="11"/>
       <c r="F85" s="6"/>
-      <c r="G85" s="162" t="s">
+      <c r="G85" s="177" t="s">
         <v>191</v>
       </c>
-      <c r="H85" s="162"/>
+      <c r="H85" s="177"/>
       <c r="I85" s="90">
         <f>AVERAGE(simPy_sheet!AJ57:AJ62)</f>
         <v>0.19999999999999998</v>
@@ -38679,24 +38539,24 @@
       <c r="AJ88" s="9"/>
     </row>
     <row r="89" spans="3:36" ht="32.4" customHeight="1">
-      <c r="C89" s="173" t="s">
+      <c r="C89" s="172" t="s">
         <v>193</v>
       </c>
-      <c r="D89" s="173"/>
-      <c r="E89" s="173"/>
-      <c r="F89" s="173"/>
-      <c r="G89" s="173"/>
-      <c r="H89" s="173"/>
-      <c r="I89" s="173"/>
-      <c r="J89" s="173"/>
-      <c r="K89" s="173"/>
-      <c r="L89" s="173"/>
-      <c r="M89" s="173"/>
-      <c r="N89" s="173"/>
-      <c r="O89" s="173"/>
-      <c r="P89" s="173"/>
-      <c r="Q89" s="173"/>
-      <c r="R89" s="173"/>
+      <c r="D89" s="172"/>
+      <c r="E89" s="172"/>
+      <c r="F89" s="172"/>
+      <c r="G89" s="172"/>
+      <c r="H89" s="172"/>
+      <c r="I89" s="172"/>
+      <c r="J89" s="172"/>
+      <c r="K89" s="172"/>
+      <c r="L89" s="172"/>
+      <c r="M89" s="172"/>
+      <c r="N89" s="172"/>
+      <c r="O89" s="172"/>
+      <c r="P89" s="172"/>
+      <c r="Q89" s="172"/>
+      <c r="R89" s="172"/>
       <c r="U89" s="83"/>
     </row>
     <row r="90" spans="3:36" ht="16.8">
@@ -38918,9 +38778,9 @@
       <c r="D95" s="11"/>
       <c r="E95" s="11"/>
       <c r="F95" s="11"/>
-      <c r="G95" s="136"/>
-      <c r="H95" s="136"/>
-      <c r="I95" s="136"/>
+      <c r="G95" s="163"/>
+      <c r="H95" s="163"/>
+      <c r="I95" s="163"/>
       <c r="J95" s="84" t="s">
         <v>19</v>
       </c>
@@ -39122,6 +38982,56 @@
     </row>
   </sheetData>
   <mergeCells count="66">
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="G52:H52"/>
+    <mergeCell ref="C57:L57"/>
+    <mergeCell ref="I59:U59"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="I47:U47"/>
+    <mergeCell ref="G47:H48"/>
+    <mergeCell ref="G59:H60"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="C45:L45"/>
+    <mergeCell ref="G53:H53"/>
+    <mergeCell ref="G54:H54"/>
+    <mergeCell ref="G95:I95"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="G81:H81"/>
+    <mergeCell ref="I73:U73"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="C89:R89"/>
+    <mergeCell ref="C72:L72"/>
+    <mergeCell ref="G74:H74"/>
+    <mergeCell ref="G75:H75"/>
+    <mergeCell ref="G76:H76"/>
+    <mergeCell ref="G83:H83"/>
+    <mergeCell ref="G84:H84"/>
+    <mergeCell ref="G85:H85"/>
+    <mergeCell ref="G77:H77"/>
+    <mergeCell ref="G61:H61"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="G62:H62"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="C35:L35"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="G36:H37"/>
+    <mergeCell ref="I36:U36"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="F22:L22"/>
+    <mergeCell ref="F23:L23"/>
+    <mergeCell ref="R23:X23"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="V25:X25"/>
+    <mergeCell ref="C18:L18"/>
+    <mergeCell ref="N18:X18"/>
+    <mergeCell ref="F20:L20"/>
+    <mergeCell ref="R20:X20"/>
+    <mergeCell ref="F21:L21"/>
+    <mergeCell ref="R21:X21"/>
     <mergeCell ref="G78:H78"/>
     <mergeCell ref="G79:H79"/>
     <mergeCell ref="G80:H80"/>
@@ -39138,56 +39048,6 @@
     <mergeCell ref="V30:X30"/>
     <mergeCell ref="T31:U31"/>
     <mergeCell ref="V31:X31"/>
-    <mergeCell ref="C18:L18"/>
-    <mergeCell ref="N18:X18"/>
-    <mergeCell ref="F20:L20"/>
-    <mergeCell ref="R20:X20"/>
-    <mergeCell ref="F21:L21"/>
-    <mergeCell ref="R21:X21"/>
-    <mergeCell ref="F22:L22"/>
-    <mergeCell ref="F23:L23"/>
-    <mergeCell ref="R23:X23"/>
-    <mergeCell ref="T25:U25"/>
-    <mergeCell ref="V25:X25"/>
-    <mergeCell ref="C35:L35"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="G36:H37"/>
-    <mergeCell ref="I36:U36"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="G61:H61"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="G62:H62"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="G95:I95"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="G81:H81"/>
-    <mergeCell ref="I73:U73"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="C89:R89"/>
-    <mergeCell ref="C72:L72"/>
-    <mergeCell ref="G74:H74"/>
-    <mergeCell ref="G75:H75"/>
-    <mergeCell ref="G76:H76"/>
-    <mergeCell ref="G83:H83"/>
-    <mergeCell ref="G84:H84"/>
-    <mergeCell ref="G85:H85"/>
-    <mergeCell ref="G77:H77"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="G52:H52"/>
-    <mergeCell ref="C57:L57"/>
-    <mergeCell ref="I59:U59"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="I47:U47"/>
-    <mergeCell ref="G47:H48"/>
-    <mergeCell ref="G59:H60"/>
-    <mergeCell ref="G50:H50"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="C45:L45"/>
-    <mergeCell ref="G53:H53"/>
-    <mergeCell ref="G54:H54"/>
   </mergeCells>
   <conditionalFormatting sqref="A75:B86 C82:S82 C83:G83 I83:S83 C84:F84 I84:U84 F85 I85:S85 F86:S86 S89 A89:B91 C90:S92 C93:E93 R93:S93 C94:S95">
     <cfRule type="expression" dxfId="9" priority="6">
@@ -39367,49 +39227,49 @@
       <c r="M15" s="6"/>
     </row>
     <row r="16" spans="3:24" ht="36.6" customHeight="1">
-      <c r="C16" s="173" t="s">
+      <c r="C16" s="172" t="s">
         <v>79</v>
       </c>
-      <c r="D16" s="173"/>
-      <c r="E16" s="173"/>
-      <c r="F16" s="173"/>
-      <c r="G16" s="173"/>
-      <c r="H16" s="173"/>
-      <c r="I16" s="173"/>
-      <c r="J16" s="173"/>
-      <c r="K16" s="173"/>
-      <c r="L16" s="173"/>
+      <c r="D16" s="172"/>
+      <c r="E16" s="172"/>
+      <c r="F16" s="172"/>
+      <c r="G16" s="172"/>
+      <c r="H16" s="172"/>
+      <c r="I16" s="172"/>
+      <c r="J16" s="172"/>
+      <c r="K16" s="172"/>
+      <c r="L16" s="172"/>
       <c r="M16" s="6"/>
-      <c r="O16" s="173" t="s">
+      <c r="O16" s="172" t="s">
         <v>29</v>
       </c>
-      <c r="P16" s="173"/>
-      <c r="Q16" s="173"/>
-      <c r="R16" s="173"/>
-      <c r="S16" s="173"/>
-      <c r="T16" s="173"/>
-      <c r="U16" s="173"/>
-      <c r="V16" s="173"/>
-      <c r="W16" s="173"/>
-      <c r="X16" s="173"/>
+      <c r="P16" s="172"/>
+      <c r="Q16" s="172"/>
+      <c r="R16" s="172"/>
+      <c r="S16" s="172"/>
+      <c r="T16" s="172"/>
+      <c r="U16" s="172"/>
+      <c r="V16" s="172"/>
+      <c r="W16" s="172"/>
+      <c r="X16" s="172"/>
     </row>
     <row r="17" spans="3:27" s="16" customFormat="1" ht="34.950000000000003" customHeight="1">
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
       <c r="F17" s="15"/>
-      <c r="G17" s="144" t="s">
+      <c r="G17" s="157" t="s">
         <v>30</v>
       </c>
-      <c r="H17" s="144"/>
-      <c r="I17" s="143" t="s">
+      <c r="H17" s="157"/>
+      <c r="I17" s="156" t="s">
         <v>31</v>
       </c>
-      <c r="J17" s="143"/>
-      <c r="K17" s="143" t="s">
+      <c r="J17" s="156"/>
+      <c r="K17" s="156" t="s">
         <v>18</v>
       </c>
-      <c r="L17" s="143"/>
+      <c r="L17" s="156"/>
       <c r="M17" s="15"/>
       <c r="O17" s="23"/>
       <c r="P17" s="23"/>
@@ -39417,14 +39277,14 @@
       <c r="R17" s="24"/>
       <c r="S17" s="24"/>
       <c r="T17" s="24"/>
-      <c r="U17" s="215" t="s">
+      <c r="U17" s="195" t="s">
         <v>30</v>
       </c>
-      <c r="V17" s="215"/>
-      <c r="W17" s="214" t="s">
+      <c r="V17" s="195"/>
+      <c r="W17" s="194" t="s">
         <v>18</v>
       </c>
-      <c r="X17" s="214"/>
+      <c r="X17" s="194"/>
       <c r="Z17" s="27" t="s">
         <v>32</v>
       </c>
@@ -39437,22 +39297,22 @@
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="183">
+      <c r="G18" s="221">
         <v>62842.05</v>
       </c>
-      <c r="H18" s="184"/>
-      <c r="I18" s="191"/>
-      <c r="J18" s="186"/>
-      <c r="K18" s="190">
+      <c r="H18" s="222"/>
+      <c r="I18" s="225"/>
+      <c r="J18" s="224"/>
+      <c r="K18" s="220">
         <f>IF(I18="", G18, I18)</f>
         <v>62842.05</v>
       </c>
-      <c r="L18" s="190"/>
+      <c r="L18" s="220"/>
       <c r="M18" s="6"/>
-      <c r="O18" s="216" t="s">
+      <c r="O18" s="198" t="s">
         <v>34</v>
       </c>
-      <c r="P18" s="217"/>
+      <c r="P18" s="199"/>
       <c r="Q18" s="33" t="s">
         <v>33</v>
       </c>
@@ -39463,11 +39323,11 @@
         <v>62842.05</v>
       </c>
       <c r="V18" s="197"/>
-      <c r="W18" s="194">
+      <c r="W18" s="186">
         <f>K18</f>
         <v>62842.05</v>
       </c>
-      <c r="X18" s="194"/>
+      <c r="X18" s="186"/>
       <c r="Z18" s="28">
         <f>U18</f>
         <v>62842.05</v>
@@ -39484,20 +39344,20 @@
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
-      <c r="G19" s="183">
+      <c r="G19" s="221">
         <v>51121.9</v>
       </c>
-      <c r="H19" s="184"/>
-      <c r="I19" s="185"/>
-      <c r="J19" s="186"/>
-      <c r="K19" s="190">
+      <c r="H19" s="222"/>
+      <c r="I19" s="223"/>
+      <c r="J19" s="224"/>
+      <c r="K19" s="220">
         <f>IF(I19="", G19, I19)</f>
         <v>51121.9</v>
       </c>
-      <c r="L19" s="190"/>
+      <c r="L19" s="220"/>
       <c r="M19" s="6"/>
-      <c r="O19" s="218"/>
-      <c r="P19" s="219"/>
+      <c r="O19" s="200"/>
+      <c r="P19" s="201"/>
       <c r="Q19" s="34" t="s">
         <v>35</v>
       </c>
@@ -39508,11 +39368,11 @@
         <v>51121.9</v>
       </c>
       <c r="V19" s="197"/>
-      <c r="W19" s="194">
+      <c r="W19" s="186">
         <f>K19</f>
         <v>51121.9</v>
       </c>
-      <c r="X19" s="194"/>
+      <c r="X19" s="186"/>
       <c r="Z19" s="28">
         <f t="shared" ref="Z19:Z27" si="0">U19</f>
         <v>51121.9</v>
@@ -39529,20 +39389,20 @@
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
-      <c r="G20" s="183">
+      <c r="G20" s="221">
         <v>39390.800000000003</v>
       </c>
-      <c r="H20" s="184"/>
-      <c r="I20" s="185"/>
-      <c r="J20" s="186"/>
-      <c r="K20" s="190">
+      <c r="H20" s="222"/>
+      <c r="I20" s="223"/>
+      <c r="J20" s="224"/>
+      <c r="K20" s="220">
         <f>IF(I20="", G20, I20)</f>
         <v>39390.800000000003</v>
       </c>
-      <c r="L20" s="190"/>
+      <c r="L20" s="220"/>
       <c r="M20" s="6"/>
-      <c r="O20" s="218"/>
-      <c r="P20" s="219"/>
+      <c r="O20" s="200"/>
+      <c r="P20" s="201"/>
       <c r="Q20" s="34" t="s">
         <v>36</v>
       </c>
@@ -39553,11 +39413,11 @@
         <v>39390.800000000003</v>
       </c>
       <c r="V20" s="197"/>
-      <c r="W20" s="194">
+      <c r="W20" s="186">
         <f>K20</f>
         <v>39390.800000000003</v>
       </c>
-      <c r="X20" s="194"/>
+      <c r="X20" s="186"/>
       <c r="Z20" s="28">
         <f t="shared" si="0"/>
         <v>39390.800000000003</v>
@@ -39574,20 +39434,20 @@
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
-      <c r="G21" s="183">
+      <c r="G21" s="221">
         <v>9004.5500000000011</v>
       </c>
-      <c r="H21" s="184"/>
-      <c r="I21" s="185"/>
-      <c r="J21" s="186"/>
-      <c r="K21" s="190">
+      <c r="H21" s="222"/>
+      <c r="I21" s="223"/>
+      <c r="J21" s="224"/>
+      <c r="K21" s="220">
         <f>IF(I21="", G21, I21)</f>
         <v>9004.5500000000011</v>
       </c>
-      <c r="L21" s="190"/>
+      <c r="L21" s="220"/>
       <c r="M21" s="6"/>
-      <c r="O21" s="220"/>
-      <c r="P21" s="221"/>
+      <c r="O21" s="202"/>
+      <c r="P21" s="203"/>
       <c r="Q21" s="128" t="s">
         <v>37</v>
       </c>
@@ -39598,11 +39458,11 @@
         <v>9004.5500000000011</v>
       </c>
       <c r="V21" s="197"/>
-      <c r="W21" s="194">
+      <c r="W21" s="186">
         <f>K21</f>
         <v>9004.5500000000011</v>
       </c>
-      <c r="X21" s="194"/>
+      <c r="X21" s="186"/>
       <c r="Z21" s="28">
         <f t="shared" si="0"/>
         <v>9004.5500000000011</v>
@@ -39616,10 +39476,10 @@
       <c r="J22" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="O22" s="202" t="s">
+      <c r="O22" s="212" t="s">
         <v>39</v>
       </c>
-      <c r="P22" s="203"/>
+      <c r="P22" s="213"/>
       <c r="Q22" s="29" t="str">
         <f>E36</f>
         <v>Intervention 1: KRT intervention</v>
@@ -39627,15 +39487,15 @@
       <c r="R22" s="29"/>
       <c r="S22" s="29"/>
       <c r="T22" s="30"/>
-      <c r="U22" s="200">
+      <c r="U22" s="210">
         <v>0</v>
       </c>
-      <c r="V22" s="201"/>
-      <c r="W22" s="194">
+      <c r="V22" s="211"/>
+      <c r="W22" s="186">
         <f t="shared" ref="W22:W27" si="2">V36</f>
         <v>0</v>
       </c>
-      <c r="X22" s="195"/>
+      <c r="X22" s="187"/>
       <c r="Z22" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -39647,8 +39507,8 @@
     </row>
     <row r="23" spans="3:27" ht="19.2" hidden="1">
       <c r="J23" s="17"/>
-      <c r="O23" s="204"/>
-      <c r="P23" s="205"/>
+      <c r="O23" s="214"/>
+      <c r="P23" s="215"/>
       <c r="Q23" s="31" t="str">
         <f>E37</f>
         <v>Intervention 2: KRT intervention</v>
@@ -39656,15 +39516,15 @@
       <c r="R23" s="31"/>
       <c r="S23" s="31"/>
       <c r="T23" s="32"/>
-      <c r="U23" s="200">
+      <c r="U23" s="210">
         <v>0</v>
       </c>
-      <c r="V23" s="201"/>
-      <c r="W23" s="194">
+      <c r="V23" s="211"/>
+      <c r="W23" s="186">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="X23" s="195"/>
+      <c r="X23" s="187"/>
       <c r="Z23" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -39676,8 +39536,8 @@
     </row>
     <row r="24" spans="3:27" ht="19.2" hidden="1">
       <c r="J24" s="17"/>
-      <c r="O24" s="204"/>
-      <c r="P24" s="205"/>
+      <c r="O24" s="214"/>
+      <c r="P24" s="215"/>
       <c r="Q24" s="31" t="str">
         <f>E38</f>
         <v>Intervention 3: KRT intervention</v>
@@ -39685,15 +39545,15 @@
       <c r="R24" s="31"/>
       <c r="S24" s="31"/>
       <c r="T24" s="32"/>
-      <c r="U24" s="200">
+      <c r="U24" s="210">
         <v>0</v>
       </c>
-      <c r="V24" s="201"/>
-      <c r="W24" s="194">
+      <c r="V24" s="211"/>
+      <c r="W24" s="186">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="X24" s="195"/>
+      <c r="X24" s="187"/>
       <c r="Z24" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -39705,8 +39565,8 @@
     </row>
     <row r="25" spans="3:27" ht="19.2" hidden="1">
       <c r="J25" s="17"/>
-      <c r="O25" s="204"/>
-      <c r="P25" s="205"/>
+      <c r="O25" s="214"/>
+      <c r="P25" s="215"/>
       <c r="Q25" s="31" t="str">
         <f>E39</f>
         <v>Intervention 4</v>
@@ -39714,15 +39574,15 @@
       <c r="R25" s="31"/>
       <c r="S25" s="31"/>
       <c r="T25" s="32"/>
-      <c r="U25" s="200">
+      <c r="U25" s="210">
         <v>0</v>
       </c>
-      <c r="V25" s="201"/>
-      <c r="W25" s="194">
+      <c r="V25" s="211"/>
+      <c r="W25" s="186">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="X25" s="195"/>
+      <c r="X25" s="187"/>
       <c r="Z25" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -39734,8 +39594,8 @@
     </row>
     <row r="26" spans="3:27" ht="19.2" hidden="1">
       <c r="J26" s="17"/>
-      <c r="O26" s="204"/>
-      <c r="P26" s="205"/>
+      <c r="O26" s="214"/>
+      <c r="P26" s="215"/>
       <c r="Q26" s="31" t="str">
         <f>E40</f>
         <v>Intervention 5</v>
@@ -39743,15 +39603,15 @@
       <c r="R26" s="31"/>
       <c r="S26" s="31"/>
       <c r="T26" s="32"/>
-      <c r="U26" s="200">
+      <c r="U26" s="210">
         <v>0</v>
       </c>
-      <c r="V26" s="201"/>
-      <c r="W26" s="194">
+      <c r="V26" s="211"/>
+      <c r="W26" s="186">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="X26" s="195"/>
+      <c r="X26" s="187"/>
       <c r="Z26" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -39762,23 +39622,23 @@
       </c>
     </row>
     <row r="27" spans="3:27" ht="19.2" hidden="1">
-      <c r="O27" s="206"/>
-      <c r="P27" s="207"/>
+      <c r="O27" s="216"/>
+      <c r="P27" s="217"/>
       <c r="Q27" s="35" t="s">
         <v>40</v>
       </c>
       <c r="R27" s="36"/>
       <c r="S27" s="36"/>
       <c r="T27" s="37"/>
-      <c r="U27" s="200">
+      <c r="U27" s="210">
         <v>0</v>
       </c>
-      <c r="V27" s="201"/>
-      <c r="W27" s="224">
+      <c r="V27" s="211"/>
+      <c r="W27" s="188">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="X27" s="225"/>
+      <c r="X27" s="189"/>
       <c r="Z27" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -39828,28 +39688,28 @@
       <c r="M30" s="11"/>
     </row>
     <row r="31" spans="3:27" ht="179.4" hidden="1" customHeight="1">
-      <c r="C31" s="193"/>
-      <c r="D31" s="193"/>
-      <c r="E31" s="193"/>
-      <c r="F31" s="193"/>
-      <c r="G31" s="193"/>
-      <c r="H31" s="193"/>
-      <c r="I31" s="193"/>
-      <c r="J31" s="193"/>
-      <c r="K31" s="193"/>
-      <c r="L31" s="193"/>
-      <c r="M31" s="193"/>
-      <c r="N31" s="193"/>
-      <c r="O31" s="193"/>
-      <c r="P31" s="193"/>
-      <c r="Q31" s="193"/>
-      <c r="R31" s="193"/>
-      <c r="S31" s="193"/>
-      <c r="T31" s="193"/>
-      <c r="U31" s="193"/>
-      <c r="V31" s="193"/>
-      <c r="W31" s="193"/>
-      <c r="X31" s="193"/>
+      <c r="C31" s="227"/>
+      <c r="D31" s="227"/>
+      <c r="E31" s="227"/>
+      <c r="F31" s="227"/>
+      <c r="G31" s="227"/>
+      <c r="H31" s="227"/>
+      <c r="I31" s="227"/>
+      <c r="J31" s="227"/>
+      <c r="K31" s="227"/>
+      <c r="L31" s="227"/>
+      <c r="M31" s="227"/>
+      <c r="N31" s="227"/>
+      <c r="O31" s="227"/>
+      <c r="P31" s="227"/>
+      <c r="Q31" s="227"/>
+      <c r="R31" s="227"/>
+      <c r="S31" s="227"/>
+      <c r="T31" s="227"/>
+      <c r="U31" s="227"/>
+      <c r="V31" s="227"/>
+      <c r="W31" s="227"/>
+      <c r="X31" s="227"/>
     </row>
     <row r="32" spans="3:27" ht="16.8" hidden="1">
       <c r="G32" s="21"/>
@@ -39868,12 +39728,12 @@
       <c r="T32" s="21"/>
     </row>
     <row r="33" spans="3:23" ht="34.950000000000003" hidden="1" customHeight="1">
-      <c r="E33" s="222" t="s">
+      <c r="E33" s="204" t="s">
         <v>42</v>
       </c>
-      <c r="F33" s="222"/>
-      <c r="G33" s="222"/>
-      <c r="H33" s="222"/>
+      <c r="F33" s="204"/>
+      <c r="G33" s="204"/>
+      <c r="H33" s="204"/>
       <c r="I33" s="20">
         <v>2023</v>
       </c>
@@ -39913,18 +39773,18 @@
       <c r="U33" s="20">
         <v>2035</v>
       </c>
-      <c r="V33" s="223" t="s">
+      <c r="V33" s="205" t="s">
         <v>43</v>
       </c>
-      <c r="W33" s="223"/>
+      <c r="W33" s="205"/>
     </row>
     <row r="34" spans="3:23" hidden="1">
-      <c r="E34" s="213" t="s">
+      <c r="E34" s="190" t="s">
         <v>44</v>
       </c>
-      <c r="F34" s="213"/>
-      <c r="G34" s="213"/>
-      <c r="H34" s="213"/>
+      <c r="F34" s="190"/>
+      <c r="G34" s="190"/>
+      <c r="H34" s="190"/>
       <c r="I34" s="39"/>
       <c r="J34" s="39"/>
       <c r="K34" s="39"/>
@@ -39944,21 +39804,21 @@
       <c r="S34" s="39"/>
       <c r="T34" s="39"/>
       <c r="U34" s="39"/>
-      <c r="V34" s="208">
+      <c r="V34" s="185">
         <f t="shared" ref="V34:V41" si="3">SUM(I34:U34)</f>
         <v>20000</v>
       </c>
-      <c r="W34" s="208"/>
+      <c r="W34" s="185"/>
     </row>
     <row r="35" spans="3:23" s="16" customFormat="1" ht="16.2" hidden="1" customHeight="1">
-      <c r="C35" s="192"/>
-      <c r="D35" s="192"/>
-      <c r="E35" s="213" t="s">
+      <c r="C35" s="226"/>
+      <c r="D35" s="226"/>
+      <c r="E35" s="190" t="s">
         <v>45</v>
       </c>
-      <c r="F35" s="213"/>
-      <c r="G35" s="213"/>
-      <c r="H35" s="213"/>
+      <c r="F35" s="190"/>
+      <c r="G35" s="190"/>
+      <c r="H35" s="190"/>
       <c r="I35" s="39"/>
       <c r="J35" s="39"/>
       <c r="K35" s="39"/>
@@ -39990,23 +39850,23 @@
       <c r="U35" s="39">
         <v>500</v>
       </c>
-      <c r="V35" s="208">
+      <c r="V35" s="185">
         <f t="shared" si="3"/>
         <v>64000</v>
       </c>
-      <c r="W35" s="208"/>
+      <c r="W35" s="185"/>
     </row>
     <row r="36" spans="3:23" hidden="1">
-      <c r="C36" s="212" t="s">
+      <c r="C36" s="206" t="s">
         <v>46</v>
       </c>
-      <c r="D36" s="212"/>
-      <c r="E36" s="187" t="s">
+      <c r="D36" s="206"/>
+      <c r="E36" s="191" t="s">
         <v>80</v>
       </c>
-      <c r="F36" s="188"/>
-      <c r="G36" s="188"/>
-      <c r="H36" s="189"/>
+      <c r="F36" s="192"/>
+      <c r="G36" s="192"/>
+      <c r="H36" s="193"/>
       <c r="I36" s="40"/>
       <c r="J36" s="40"/>
       <c r="K36" s="40"/>
@@ -40020,23 +39880,23 @@
       <c r="S36" s="38"/>
       <c r="T36" s="38"/>
       <c r="U36" s="38"/>
-      <c r="V36" s="209">
+      <c r="V36" s="218">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="W36" s="210"/>
+      <c r="W36" s="219"/>
     </row>
     <row r="37" spans="3:23" hidden="1">
-      <c r="C37" s="211" t="s">
+      <c r="C37" s="207" t="s">
         <v>47</v>
       </c>
-      <c r="D37" s="211"/>
-      <c r="E37" s="187" t="s">
+      <c r="D37" s="207"/>
+      <c r="E37" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="F37" s="188"/>
-      <c r="G37" s="188"/>
-      <c r="H37" s="189"/>
+      <c r="F37" s="192"/>
+      <c r="G37" s="192"/>
+      <c r="H37" s="193"/>
       <c r="I37" s="38"/>
       <c r="J37" s="38"/>
       <c r="K37" s="38"/>
@@ -40050,23 +39910,23 @@
       <c r="S37" s="38"/>
       <c r="T37" s="38"/>
       <c r="U37" s="38"/>
-      <c r="V37" s="208">
+      <c r="V37" s="185">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="W37" s="208"/>
+      <c r="W37" s="185"/>
     </row>
     <row r="38" spans="3:23" hidden="1">
-      <c r="C38" s="211" t="s">
+      <c r="C38" s="207" t="s">
         <v>48</v>
       </c>
-      <c r="D38" s="211"/>
-      <c r="E38" s="187" t="s">
+      <c r="D38" s="207"/>
+      <c r="E38" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="F38" s="188"/>
-      <c r="G38" s="188"/>
-      <c r="H38" s="189"/>
+      <c r="F38" s="192"/>
+      <c r="G38" s="192"/>
+      <c r="H38" s="193"/>
       <c r="I38" s="38"/>
       <c r="J38" s="38"/>
       <c r="K38" s="38"/>
@@ -40080,23 +39940,23 @@
       <c r="S38" s="38"/>
       <c r="T38" s="38"/>
       <c r="U38" s="38"/>
-      <c r="V38" s="208">
+      <c r="V38" s="185">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="W38" s="208"/>
+      <c r="W38" s="185"/>
     </row>
     <row r="39" spans="3:23" ht="15" hidden="1" customHeight="1">
-      <c r="C39" s="211" t="s">
+      <c r="C39" s="207" t="s">
         <v>49</v>
       </c>
-      <c r="D39" s="211"/>
-      <c r="E39" s="187" t="s">
+      <c r="D39" s="207"/>
+      <c r="E39" s="191" t="s">
         <v>49</v>
       </c>
-      <c r="F39" s="188"/>
-      <c r="G39" s="188"/>
-      <c r="H39" s="189"/>
+      <c r="F39" s="192"/>
+      <c r="G39" s="192"/>
+      <c r="H39" s="193"/>
       <c r="I39" s="38"/>
       <c r="J39" s="38"/>
       <c r="K39" s="38"/>
@@ -40110,23 +39970,23 @@
       <c r="S39" s="38"/>
       <c r="T39" s="38"/>
       <c r="U39" s="38"/>
-      <c r="V39" s="208">
+      <c r="V39" s="185">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="W39" s="208"/>
+      <c r="W39" s="185"/>
     </row>
     <row r="40" spans="3:23" ht="15" hidden="1" customHeight="1">
-      <c r="C40" s="211" t="s">
+      <c r="C40" s="207" t="s">
         <v>50</v>
       </c>
-      <c r="D40" s="211"/>
-      <c r="E40" s="187" t="s">
+      <c r="D40" s="207"/>
+      <c r="E40" s="191" t="s">
         <v>50</v>
       </c>
-      <c r="F40" s="188"/>
-      <c r="G40" s="188"/>
-      <c r="H40" s="189"/>
+      <c r="F40" s="192"/>
+      <c r="G40" s="192"/>
+      <c r="H40" s="193"/>
       <c r="I40" s="38"/>
       <c r="J40" s="38"/>
       <c r="K40" s="38"/>
@@ -40140,23 +40000,23 @@
       <c r="S40" s="38"/>
       <c r="T40" s="38"/>
       <c r="U40" s="38"/>
-      <c r="V40" s="208">
+      <c r="V40" s="185">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="W40" s="208"/>
+      <c r="W40" s="185"/>
     </row>
     <row r="41" spans="3:23" hidden="1">
-      <c r="C41" s="198" t="s">
+      <c r="C41" s="208" t="s">
         <v>72</v>
       </c>
-      <c r="D41" s="198"/>
-      <c r="E41" s="199" t="s">
+      <c r="D41" s="208"/>
+      <c r="E41" s="209" t="s">
         <v>51</v>
       </c>
-      <c r="F41" s="199"/>
-      <c r="G41" s="199"/>
-      <c r="H41" s="199"/>
+      <c r="F41" s="209"/>
+      <c r="G41" s="209"/>
+      <c r="H41" s="209"/>
       <c r="I41" s="22">
         <f>SUM(I36:I38)</f>
         <v>0</v>
@@ -40209,11 +40069,11 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="V41" s="208">
+      <c r="V41" s="185">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="W41" s="208"/>
+      <c r="W41" s="185"/>
     </row>
     <row r="44" spans="3:23" ht="16.8">
       <c r="E44" s="26"/>
@@ -40405,12 +40265,51 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="wstTatVdFSRAf0DuE//XV2ckjyh7Er1M6yYDa8/3BPE0Ezc0ZztZK5DLucvF8Caot75oy71gerI52M8dBh3vag==" saltValue="jAFKtc8z6aub6EDLT2Imgg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="67">
-    <mergeCell ref="V34:W34"/>
-    <mergeCell ref="W23:X23"/>
-    <mergeCell ref="W24:X24"/>
-    <mergeCell ref="W25:X25"/>
-    <mergeCell ref="W26:X26"/>
-    <mergeCell ref="W27:X27"/>
+    <mergeCell ref="C16:L16"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="E38:H38"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C31:X31"/>
+    <mergeCell ref="W22:X22"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:H41"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="O22:P27"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="V40:W40"/>
+    <mergeCell ref="V41:W41"/>
+    <mergeCell ref="V35:W35"/>
+    <mergeCell ref="V36:W36"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E39:H39"/>
+    <mergeCell ref="E40:H40"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="V37:W37"/>
+    <mergeCell ref="V38:W38"/>
+    <mergeCell ref="V39:W39"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E37:H37"/>
     <mergeCell ref="E35:H35"/>
     <mergeCell ref="E36:H36"/>
     <mergeCell ref="W20:X20"/>
@@ -40427,51 +40326,12 @@
     <mergeCell ref="E33:H33"/>
     <mergeCell ref="V33:W33"/>
     <mergeCell ref="E34:H34"/>
-    <mergeCell ref="E40:H40"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="V37:W37"/>
-    <mergeCell ref="V38:W38"/>
-    <mergeCell ref="V39:W39"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E37:H37"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:H41"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="O22:P27"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="U27:V27"/>
-    <mergeCell ref="V40:W40"/>
-    <mergeCell ref="V41:W41"/>
-    <mergeCell ref="V35:W35"/>
-    <mergeCell ref="V36:W36"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E39:H39"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="C16:L16"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="E38:H38"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C31:X31"/>
-    <mergeCell ref="W22:X22"/>
+    <mergeCell ref="V34:W34"/>
+    <mergeCell ref="W23:X23"/>
+    <mergeCell ref="W24:X24"/>
+    <mergeCell ref="W25:X25"/>
+    <mergeCell ref="W26:X26"/>
+    <mergeCell ref="W27:X27"/>
   </mergeCells>
   <phoneticPr fontId="23" type="noConversion"/>
   <conditionalFormatting sqref="J22:M26">
@@ -40514,6 +40374,25 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3b4031e-841f-46f6-bede-a60d28c4ce79">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="25f82bdf-59aa-449e-b461-28a7236b0743" xsi:nil="true"/>
+    <Modifiedtime xmlns="c3b4031e-841f-46f6-bede-a60d28c4ce79" xsi:nil="true"/>
+    <BidAuthors xmlns="c3b4031e-841f-46f6-bede-a60d28c4ce79">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </BidAuthors>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F00E7D3C5223B647BCF0704F4FD63FF8" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1fa9e41d02e9b02fc955bd1400030d11">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3b4031e-841f-46f6-bede-a60d28c4ce79" xmlns:ns3="25f82bdf-59aa-449e-b461-28a7236b0743" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ce80f9b71fe371980485e1a61dbeb78d" ns2:_="" ns3:_="">
     <xsd:import namespace="c3b4031e-841f-46f6-bede-a60d28c4ce79"/>
@@ -40794,25 +40673,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3b4031e-841f-46f6-bede-a60d28c4ce79">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="25f82bdf-59aa-449e-b461-28a7236b0743" xsi:nil="true"/>
-    <Modifiedtime xmlns="c3b4031e-841f-46f6-bede-a60d28c4ce79" xsi:nil="true"/>
-    <BidAuthors xmlns="c3b4031e-841f-46f6-bede-a60d28c4ce79">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </BidAuthors>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AB1A394-CDD1-412D-97FA-5861127EE7E9}">
   <ds:schemaRefs>
@@ -40822,6 +40682,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92445AFB-1516-4879-B465-5E6529C74BBB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c3b4031e-841f-46f6-bede-a60d28c4ce79"/>
+    <ds:schemaRef ds:uri="25f82bdf-59aa-449e-b461-28a7236b0743"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98A79971-7DA6-46C3-A409-B57248166160}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -40838,15 +40709,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92445AFB-1516-4879-B465-5E6529C74BBB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c3b4031e-841f-46f6-bede-a60d28c4ce79"/>
-    <ds:schemaRef ds:uri="25f82bdf-59aa-449e-b461-28a7236b0743"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>